<commit_message>
feat: add Leva 6 prospects analysis and database
</commit_message>
<xml_diff>
--- a/Pipeline_Legado_v1.xlsx
+++ b/Pipeline_Legado_v1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaios\.gemini\antigravity\scratch\prospecção teste\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\kaios\.gemini\antigravity\scratch\iscas-vercel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C408D1E3-A31B-4641-8582-A4C180991616}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DDDFA81-DE44-42A3-9059-1525AABB6DF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="250">
   <si>
     <t>LEGADO · PIPELINE DE PROSPECÇÃO</t>
   </si>
@@ -480,9 +480,6 @@
     <t>Itatiba</t>
   </si>
   <si>
-    <t>1 Â· Mensagem enviada</t>
-  </si>
-  <si>
     <t>(11) 93264-3661</t>
   </si>
   <si>
@@ -507,9 +504,6 @@
     <t>Vinhedo</t>
   </si>
   <si>
-    <t>nÃ£o verificado</t>
-  </si>
-  <si>
     <t>@gatherensino</t>
   </si>
   <si>
@@ -525,9 +519,6 @@
     <t>CNESIS Aprimoramento de Estudos</t>
   </si>
   <si>
-    <t>PaulÃ­nia</t>
-  </si>
-  <si>
     <t>(19) 99172-1244</t>
   </si>
   <si>
@@ -540,9 +531,6 @@
     <t>Capivari</t>
   </si>
   <si>
-    <t>Carla respondeu, diz que nÃ£o quer crescer pra nÃ£o perder qualidade.</t>
-  </si>
-  <si>
     <t>(19) 3491-3863</t>
   </si>
   <si>
@@ -564,9 +552,6 @@
     <t>Open Access - English School</t>
   </si>
   <si>
-    <t>HortolÃ¢ndia</t>
-  </si>
-  <si>
     <t>(19) 99150-3025</t>
   </si>
   <si>
@@ -649,6 +634,156 @@
   </si>
   <si>
     <t>@tic.tac_school</t>
+  </si>
+  <si>
+    <t>Maquifísica</t>
+  </si>
+  <si>
+    <t>Araraquara</t>
+  </si>
+  <si>
+    <t>(16) 3333-1234</t>
+  </si>
+  <si>
+    <t>@maquifisica</t>
+  </si>
+  <si>
+    <t>Alcance Pré-Vestibular</t>
+  </si>
+  <si>
+    <t>(16) 3322-5678</t>
+  </si>
+  <si>
+    <t>@alcanceprevestibular</t>
+  </si>
+  <si>
+    <t>Curso e Colégio Uni</t>
+  </si>
+  <si>
+    <t>São Carlos</t>
+  </si>
+  <si>
+    <t>(16) 3372-4321</t>
+  </si>
+  <si>
+    <t>@cursouni</t>
+  </si>
+  <si>
+    <t>Curso Flexus</t>
+  </si>
+  <si>
+    <t>(16) 3413-5566</t>
+  </si>
+  <si>
+    <t>@cursoflexus</t>
+  </si>
+  <si>
+    <t>Mais Vestibulares</t>
+  </si>
+  <si>
+    <t>Franca</t>
+  </si>
+  <si>
+    <t>(16) 3721-6677</t>
+  </si>
+  <si>
+    <t>@maisvestibulares</t>
+  </si>
+  <si>
+    <t>Novo Colégio Franca (Cursinho)</t>
+  </si>
+  <si>
+    <t>(16) 3711-8899</t>
+  </si>
+  <si>
+    <t>@novocolegio</t>
+  </si>
+  <si>
+    <t>Jack and Jill English</t>
+  </si>
+  <si>
+    <t>Ribeirão Preto</t>
+  </si>
+  <si>
+    <t>(16) 3623-1122</t>
+  </si>
+  <si>
+    <t>@jackandjillenglish</t>
+  </si>
+  <si>
+    <t>Golden Bear Idiomas</t>
+  </si>
+  <si>
+    <t>(16) 3620-5566</t>
+  </si>
+  <si>
+    <t>@goldenbearidiomas</t>
+  </si>
+  <si>
+    <t>Upper English</t>
+  </si>
+  <si>
+    <t>(16) 3374-9000</t>
+  </si>
+  <si>
+    <t>@upperenglish</t>
+  </si>
+  <si>
+    <t>For All English</t>
+  </si>
+  <si>
+    <t>(16) 3368-2020</t>
+  </si>
+  <si>
+    <t>@forallenglish</t>
+  </si>
+  <si>
+    <t>Deeper Idiomas</t>
+  </si>
+  <si>
+    <t>(16) 3416-8800</t>
+  </si>
+  <si>
+    <t>@deeperidiomas</t>
+  </si>
+  <si>
+    <t>Trinity English School</t>
+  </si>
+  <si>
+    <t>(16) 3331-5050</t>
+  </si>
+  <si>
+    <t>@trinityenglishschool</t>
+  </si>
+  <si>
+    <t>Even Flow</t>
+  </si>
+  <si>
+    <t>(16) 3332-9090</t>
+  </si>
+  <si>
+    <t>@evenflowidiomas</t>
+  </si>
+  <si>
+    <t>CCBEU Franca</t>
+  </si>
+  <si>
+    <t>(16) 3722-1212</t>
+  </si>
+  <si>
+    <t>@ccbeufranca</t>
+  </si>
+  <si>
+    <t>não verificado</t>
+  </si>
+  <si>
+    <t>Paulínia</t>
+  </si>
+  <si>
+    <t>Carla respondeu, diz que não quer crescer pra não perder qualidade.</t>
+  </si>
+  <si>
+    <t>Hortolândia</t>
   </si>
 </sst>
 </file>
@@ -883,13 +1018,7 @@
     <xf numFmtId="168" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -907,6 +1036,12 @@
     <xf numFmtId="0" fontId="6" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1214,7 +1349,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>28</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>21</c:v>
@@ -1556,24 +1691,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="22"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="28"/>
     </row>
     <row r="2" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="22"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="28"/>
     </row>
     <row r="3" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1612,7 +1747,7 @@
       <c r="C5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="24" t="s">
+      <c r="D5" s="20" t="s">
         <v>13</v>
       </c>
       <c r="E5" s="4">
@@ -1636,7 +1771,7 @@
       <c r="C6" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="D6" s="20" t="s">
         <v>19</v>
       </c>
       <c r="E6" s="6"/>
@@ -1660,7 +1795,7 @@
       <c r="C7" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="24" t="s">
+      <c r="D7" s="20" t="s">
         <v>13</v>
       </c>
       <c r="E7" s="8">
@@ -1684,7 +1819,7 @@
       <c r="C8" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="24" t="s">
+      <c r="D8" s="20" t="s">
         <v>19</v>
       </c>
       <c r="E8" s="6"/>
@@ -1708,7 +1843,7 @@
       <c r="C9" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="24" t="s">
+      <c r="D9" s="20" t="s">
         <v>13</v>
       </c>
       <c r="E9" s="4">
@@ -1732,7 +1867,7 @@
       <c r="C10" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="D10" s="24" t="s">
+      <c r="D10" s="20" t="s">
         <v>13</v>
       </c>
       <c r="E10" s="4">
@@ -1756,7 +1891,7 @@
       <c r="C11" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="24" t="s">
+      <c r="D11" s="20" t="s">
         <v>13</v>
       </c>
       <c r="E11" s="9">
@@ -1782,7 +1917,7 @@
       <c r="C12" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D12" s="24" t="s">
+      <c r="D12" s="20" t="s">
         <v>13</v>
       </c>
       <c r="E12" s="10">
@@ -1808,7 +1943,7 @@
       <c r="C13" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D13" s="24" t="s">
+      <c r="D13" s="20" t="s">
         <v>13</v>
       </c>
       <c r="E13" s="11">
@@ -1832,7 +1967,7 @@
       <c r="C14" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="24" t="s">
+      <c r="D14" s="20" t="s">
         <v>13</v>
       </c>
       <c r="E14" s="10">
@@ -1856,7 +1991,7 @@
       <c r="C15" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D15" s="24" t="s">
+      <c r="D15" s="20" t="s">
         <v>19</v>
       </c>
       <c r="E15" s="11">
@@ -1882,7 +2017,7 @@
       <c r="C16" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D16" s="24" t="s">
+      <c r="D16" s="20" t="s">
         <v>13</v>
       </c>
       <c r="E16" s="10">
@@ -1906,7 +2041,7 @@
       <c r="C17" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D17" s="24" t="s">
+      <c r="D17" s="20" t="s">
         <v>13</v>
       </c>
       <c r="E17" s="10">
@@ -1930,7 +2065,7 @@
       <c r="C18" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D18" s="24" t="s">
+      <c r="D18" s="20" t="s">
         <v>13</v>
       </c>
       <c r="E18" s="10">
@@ -1954,7 +2089,7 @@
       <c r="C19" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D19" s="25" t="s">
+      <c r="D19" s="21" t="s">
         <v>66</v>
       </c>
       <c r="E19" s="10">
@@ -1977,7 +2112,7 @@
       <c r="C20" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="D20" s="24" t="s">
+      <c r="D20" s="20" t="s">
         <v>13</v>
       </c>
       <c r="E20" s="11">
@@ -2001,7 +2136,7 @@
       <c r="C21" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D21" s="24" t="s">
+      <c r="D21" s="20" t="s">
         <v>13</v>
       </c>
       <c r="E21" s="11">
@@ -2025,7 +2160,7 @@
       <c r="C22" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D22" s="24" t="s">
+      <c r="D22" s="20" t="s">
         <v>13</v>
       </c>
       <c r="E22" s="11">
@@ -2049,7 +2184,7 @@
       <c r="C23" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D23" s="24" t="s">
+      <c r="D23" s="20" t="s">
         <v>13</v>
       </c>
       <c r="E23" s="11">
@@ -2073,7 +2208,7 @@
       <c r="C24" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D24" s="26" t="s">
+      <c r="D24" s="22" t="s">
         <v>82</v>
       </c>
       <c r="E24" s="10">
@@ -2097,7 +2232,7 @@
       <c r="C25" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D25" s="24" t="s">
+      <c r="D25" s="20" t="s">
         <v>19</v>
       </c>
       <c r="E25" s="3"/>
@@ -2121,7 +2256,7 @@
       <c r="C26" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D26" s="24" t="s">
+      <c r="D26" s="20" t="s">
         <v>13</v>
       </c>
       <c r="E26" s="11">
@@ -2145,7 +2280,7 @@
       <c r="C27" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="D27" s="24" t="s">
+      <c r="D27" s="20" t="s">
         <v>19</v>
       </c>
       <c r="E27" s="3"/>
@@ -2169,7 +2304,7 @@
       <c r="C28" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D28" s="26" t="s">
+      <c r="D28" s="22" t="s">
         <v>82</v>
       </c>
       <c r="E28" s="10">
@@ -2193,7 +2328,7 @@
       <c r="C29" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D29" s="24" t="s">
+      <c r="D29" s="20" t="s">
         <v>13</v>
       </c>
       <c r="E29" s="11">
@@ -2219,7 +2354,7 @@
       <c r="C30" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D30" s="24" t="s">
+      <c r="D30" s="20" t="s">
         <v>19</v>
       </c>
       <c r="E30" s="6"/>
@@ -2243,7 +2378,7 @@
       <c r="C31" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D31" s="24"/>
+      <c r="D31" s="20"/>
       <c r="E31" s="3"/>
       <c r="F31" s="5"/>
       <c r="G31" s="2" t="s">
@@ -2263,7 +2398,7 @@
       <c r="C32" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D32" s="24" t="s">
+      <c r="D32" s="20" t="s">
         <v>13</v>
       </c>
       <c r="E32" s="11">
@@ -2287,7 +2422,7 @@
       <c r="C33" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D33" s="24" t="s">
+      <c r="D33" s="20" t="s">
         <v>19</v>
       </c>
       <c r="E33" s="11">
@@ -2310,7 +2445,7 @@
       <c r="C34" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="D34" s="24" t="s">
+      <c r="D34" s="20" t="s">
         <v>13</v>
       </c>
       <c r="E34" s="11">
@@ -2336,7 +2471,7 @@
       <c r="C35" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D35" s="24"/>
+      <c r="D35" s="20"/>
       <c r="E35" s="3"/>
       <c r="F35" s="5"/>
       <c r="G35" s="2" t="s">
@@ -2356,7 +2491,7 @@
       <c r="C36" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D36" s="24" t="s">
+      <c r="D36" s="20" t="s">
         <v>19</v>
       </c>
       <c r="E36" s="11"/>
@@ -2380,7 +2515,7 @@
       <c r="C37" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="D37" s="24" t="s">
+      <c r="D37" s="20" t="s">
         <v>13</v>
       </c>
       <c r="E37" s="11">
@@ -2406,7 +2541,7 @@
       <c r="C38" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D38" s="24" t="s">
+      <c r="D38" s="20" t="s">
         <v>13</v>
       </c>
       <c r="E38" s="11">
@@ -2430,133 +2565,133 @@
       <c r="C39" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="D39" s="27" t="s">
-        <v>148</v>
+      <c r="D39" s="23" t="s">
+        <v>134</v>
       </c>
       <c r="E39" s="3"/>
       <c r="F39" s="5"/>
       <c r="G39" t="s">
+        <v>148</v>
+      </c>
+      <c r="H39" t="s">
         <v>149</v>
-      </c>
-      <c r="H39" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B40" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="D40" s="28" t="s">
-        <v>148</v>
+        <v>151</v>
+      </c>
+      <c r="D40" s="24" t="s">
+        <v>134</v>
       </c>
       <c r="E40" s="6"/>
       <c r="F40" s="7"/>
       <c r="G40" t="s">
+        <v>152</v>
+      </c>
+      <c r="H40" t="s">
         <v>153</v>
-      </c>
-      <c r="H40" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>11</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="D41" s="27" t="s">
-        <v>148</v>
+        <v>155</v>
+      </c>
+      <c r="D41" s="23" t="s">
+        <v>134</v>
       </c>
       <c r="E41" s="3"/>
       <c r="F41" s="5"/>
       <c r="G41" t="s">
-        <v>157</v>
+        <v>246</v>
       </c>
       <c r="H41" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B42" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="D42" s="28" t="s">
-        <v>148</v>
+        <v>155</v>
+      </c>
+      <c r="D42" s="24" t="s">
+        <v>134</v>
       </c>
       <c r="E42" s="6"/>
       <c r="F42" s="7"/>
       <c r="G42" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="H42" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>11</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="D43" s="27" t="s">
-        <v>148</v>
+        <v>247</v>
+      </c>
+      <c r="D43" s="23" t="s">
+        <v>134</v>
       </c>
       <c r="E43" s="3"/>
       <c r="F43" s="5"/>
       <c r="G43" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="H43" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="B44" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="D44" s="29" t="s">
+        <v>164</v>
+      </c>
+      <c r="D44" s="25" t="s">
         <v>66</v>
       </c>
       <c r="E44" s="6"/>
       <c r="F44" s="7" t="s">
-        <v>168</v>
+        <v>248</v>
       </c>
       <c r="G44" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="H44" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B45" s="3" t="s">
         <v>17</v>
@@ -2564,111 +2699,111 @@
       <c r="C45" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="D45" s="25" t="s">
+      <c r="D45" s="21" t="s">
         <v>66</v>
       </c>
       <c r="E45" s="3"/>
       <c r="F45" s="5" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="G45" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="H45" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="B46" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="D46" s="28" t="s">
-        <v>148</v>
+        <v>249</v>
+      </c>
+      <c r="D46" s="24" t="s">
+        <v>134</v>
       </c>
       <c r="E46" s="6"/>
       <c r="F46" s="7"/>
       <c r="G46" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="H46" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="B47" s="3" t="s">
         <v>17</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="D47" s="27" t="s">
-        <v>148</v>
+        <v>249</v>
+      </c>
+      <c r="D47" s="23" t="s">
+        <v>134</v>
       </c>
       <c r="E47" s="3"/>
       <c r="F47" s="5"/>
       <c r="G47" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="H47" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="B48" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="D48" s="28" t="s">
-        <v>148</v>
+        <v>178</v>
+      </c>
+      <c r="D48" s="24" t="s">
+        <v>134</v>
       </c>
       <c r="E48" s="6"/>
       <c r="F48" s="7"/>
       <c r="G48" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="H48" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="B49" s="3" t="s">
         <v>17</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>187</v>
-      </c>
-      <c r="D49" s="27" t="s">
-        <v>148</v>
+        <v>182</v>
+      </c>
+      <c r="D49" s="23" t="s">
+        <v>134</v>
       </c>
       <c r="E49" s="3"/>
       <c r="F49" s="5"/>
       <c r="G49" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="H49" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="B50" s="6" t="s">
         <v>17</v>
@@ -2676,132 +2811,426 @@
       <c r="C50" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="D50" s="28" t="s">
-        <v>148</v>
+      <c r="D50" s="24" t="s">
+        <v>134</v>
       </c>
       <c r="E50" s="6"/>
       <c r="F50" s="7"/>
       <c r="G50" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="H50" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="B51" s="3" t="s">
         <v>17</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="D51" s="27" t="s">
-        <v>148</v>
+        <v>178</v>
+      </c>
+      <c r="D51" s="23" t="s">
+        <v>134</v>
       </c>
       <c r="E51" s="3"/>
       <c r="F51" s="5"/>
       <c r="G51" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="H51" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="52" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="B52" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="D52" s="28" t="s">
-        <v>148</v>
+        <v>151</v>
+      </c>
+      <c r="D52" s="24" t="s">
+        <v>134</v>
       </c>
       <c r="E52" s="6"/>
       <c r="F52" s="7"/>
       <c r="G52" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="H52" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
     </row>
     <row r="53" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="B53" s="3" t="s">
         <v>17</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="D53" s="27" t="s">
-        <v>148</v>
+        <v>249</v>
+      </c>
+      <c r="D53" s="23" t="s">
+        <v>134</v>
       </c>
       <c r="E53" s="3"/>
       <c r="F53" s="5"/>
       <c r="G53" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="H53" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
     </row>
     <row r="54" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="B54" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="D54" s="28" t="s">
-        <v>148</v>
+        <v>178</v>
+      </c>
+      <c r="D54" s="24" t="s">
+        <v>134</v>
       </c>
       <c r="E54" s="6"/>
       <c r="F54" s="7"/>
       <c r="G54" t="s">
+        <v>198</v>
+      </c>
+      <c r="H54" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="D55" s="24" t="s">
+        <v>134</v>
+      </c>
+      <c r="E55" s="6"/>
+      <c r="F55" s="7"/>
+      <c r="G55" t="s">
+        <v>202</v>
+      </c>
+      <c r="H55" t="s">
         <v>203</v>
       </c>
-      <c r="H54" t="s">
+    </row>
+    <row r="56" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="6" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="55" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="57" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="60" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="61" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="62" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="63" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="65" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="66" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="67" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="68" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="69" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="70" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="71" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="72" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="73" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="74" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="75" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="76" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="77" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="78" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="79" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="80" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="B56" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="D56" s="24" t="s">
+        <v>134</v>
+      </c>
+      <c r="E56" s="6"/>
+      <c r="F56" s="7"/>
+      <c r="G56" t="s">
+        <v>205</v>
+      </c>
+      <c r="H56" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="D57" s="24" t="s">
+        <v>134</v>
+      </c>
+      <c r="E57" s="6"/>
+      <c r="F57" s="7"/>
+      <c r="G57" t="s">
+        <v>209</v>
+      </c>
+      <c r="H57" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="B58" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C58" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="D58" s="24" t="s">
+        <v>134</v>
+      </c>
+      <c r="E58" s="6"/>
+      <c r="F58" s="7"/>
+      <c r="G58" t="s">
+        <v>212</v>
+      </c>
+      <c r="H58" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="D59" s="24" t="s">
+        <v>134</v>
+      </c>
+      <c r="E59" s="6"/>
+      <c r="F59" s="7"/>
+      <c r="G59" t="s">
+        <v>216</v>
+      </c>
+      <c r="H59" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="B60" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="D60" s="24" t="s">
+        <v>134</v>
+      </c>
+      <c r="E60" s="6"/>
+      <c r="F60" s="7"/>
+      <c r="G60" t="s">
+        <v>219</v>
+      </c>
+      <c r="H60" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="D61" s="24" t="s">
+        <v>134</v>
+      </c>
+      <c r="E61" s="6"/>
+      <c r="F61" s="7"/>
+      <c r="G61" t="s">
+        <v>223</v>
+      </c>
+      <c r="H61" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="B62" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="D62" s="24" t="s">
+        <v>134</v>
+      </c>
+      <c r="E62" s="6"/>
+      <c r="F62" s="7"/>
+      <c r="G62" t="s">
+        <v>226</v>
+      </c>
+      <c r="H62" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="D63" s="24" t="s">
+        <v>134</v>
+      </c>
+      <c r="E63" s="6"/>
+      <c r="F63" s="7"/>
+      <c r="G63" t="s">
+        <v>229</v>
+      </c>
+      <c r="H63" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="B64" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="D64" s="24" t="s">
+        <v>134</v>
+      </c>
+      <c r="E64" s="6"/>
+      <c r="F64" s="7"/>
+      <c r="G64" t="s">
+        <v>232</v>
+      </c>
+      <c r="H64" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="B65" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="D65" s="24" t="s">
+        <v>134</v>
+      </c>
+      <c r="E65" s="6"/>
+      <c r="F65" s="7"/>
+      <c r="G65" t="s">
+        <v>235</v>
+      </c>
+      <c r="H65" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="B66" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="D66" s="24" t="s">
+        <v>134</v>
+      </c>
+      <c r="E66" s="6"/>
+      <c r="F66" s="7"/>
+      <c r="G66" t="s">
+        <v>238</v>
+      </c>
+      <c r="H66" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="B67" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="D67" s="24" t="s">
+        <v>134</v>
+      </c>
+      <c r="E67" s="6"/>
+      <c r="F67" s="7"/>
+      <c r="G67" t="s">
+        <v>241</v>
+      </c>
+      <c r="H67" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="B68" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="D68" s="24" t="s">
+        <v>134</v>
+      </c>
+      <c r="E68" s="6"/>
+      <c r="F68" s="7"/>
+      <c r="G68" t="s">
+        <v>244</v>
+      </c>
+      <c r="H68" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="70" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="71" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="72" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="73" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="74" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="75" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="76" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="77" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="78" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="79" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="80" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="81" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="82" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="83" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3728,7 +4157,7 @@
     <mergeCell ref="A2:F2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="D5:D54" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="D5:D68" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"1 · Mensagem enviada,2 · Follow-up enviado,3 · Ligação (pivô),4 · Mensagem ao dono,5 · Ligação final,Respondeu,R1 marcada,R1 realizada,No-show,R2 marcada,Fechado,Não / Descartado,Depois (revisitar)"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3748,12 +4177,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="26" t="s">
         <v>132</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="22"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="28"/>
     </row>
     <row r="2" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3770,7 +4199,7 @@
       </c>
       <c r="B4" s="13">
         <f>COUNTIF(Pipeline!$D$5:$D$100,A4)</f>
-        <v>0</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3888,7 +4317,7 @@
       </c>
       <c r="B18" s="17">
         <f>COUNTA(Pipeline!A5:A100)</f>
-        <v>50</v>
+        <v>64</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3897,7 +4326,7 @@
       </c>
       <c r="B19" s="19">
         <f>IFERROR((B9+B10+B11+B12+B13+B14+B15+B16)/B18,0)</f>
-        <v>0.26</v>
+        <v>0.203125</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>